<commit_message>
Clean up script comments and fix missing row labels in exported results
</commit_message>
<xml_diff>
--- a/state_farm_chainladder_results.xlsx
+++ b/state_farm_chainladder_results.xlsx
@@ -14,7 +14,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+  <si>
+    <t xml:space="preserve"/>
+  </si>
   <si>
     <t xml:space="preserve">Latest</t>
   </si>
@@ -34,37 +37,82 @@
     <t xml:space="preserve">CV(IBNR)</t>
   </si>
   <si>
-    <t xml:space="preserve"/>
+    <t xml:space="preserve">1998</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1999</t>
   </si>
   <si>
     <t xml:space="preserve">0.112609817599115</t>
   </si>
   <si>
+    <t xml:space="preserve">2000</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.108328877981905</t>
   </si>
   <si>
+    <t xml:space="preserve">2001</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.0527443233111386</t>
   </si>
   <si>
+    <t xml:space="preserve">2002</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.0384381269993544</t>
   </si>
   <si>
+    <t xml:space="preserve">2003</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.0273469655957588</t>
   </si>
   <si>
+    <t xml:space="preserve">2004</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.0273207922231962</t>
   </si>
   <si>
+    <t xml:space="preserve">2005</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.0379411991930166</t>
   </si>
   <si>
+    <t xml:space="preserve">2006</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.0433909016288438</t>
   </si>
   <si>
+    <t xml:space="preserve">2007</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.041141827907498</t>
   </si>
   <si>
     <t xml:space="preserve">Totals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latest:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dev:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ultimate:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IBNR:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mack S.E.:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CV(IBNR):</t>
   </si>
   <si>
     <t xml:space="preserve">ActualUltimate</t>
@@ -421,205 +469,238 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="n">
         <v>10012517</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>10012517</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="s">
-        <v>6</v>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="n">
         <v>10283286</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>0.998326294976578</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>10300526.0421807</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>17240.0421806891</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>1941.39800536844</v>
       </c>
-      <c r="F3" t="s">
-        <v>7</v>
+      <c r="G3" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="n">
         <v>10981123</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>0.995761637387273</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>11027863.0825875</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>46740.0825875085</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>5063.30070348638</v>
       </c>
-      <c r="F4" t="s">
-        <v>8</v>
+      <c r="G4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
         <v>11837901</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>0.991073866095176</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>11944519.3794094</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>106618.379409375</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>5623.5142744777</v>
       </c>
-      <c r="F5" t="s">
-        <v>9</v>
+      <c r="G5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="n">
         <v>12490512</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>0.981641268511941</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>12724110.5286193</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>233598.528619304</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>8979.08990993114</v>
       </c>
-      <c r="F6" t="s">
-        <v>10</v>
+      <c r="G6" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="n">
         <v>11561287</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>0.963171627924413</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>12003350.8720704</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>442063.872070435</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>12089.1055006381</v>
       </c>
-      <c r="F7" t="s">
-        <v>11</v>
+      <c r="G7" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="n">
         <v>10710159</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>0.925130984191426</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>11576910.9272249</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>866751.927224856</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>23680.3493127652</v>
       </c>
-      <c r="F8" t="s">
-        <v>12</v>
+      <c r="G8" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="n">
         <v>9772146</v>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>0.853986174753088</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>11442979.159265</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>1670833.15926497</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>63393.4137139695</v>
       </c>
-      <c r="F9" t="s">
-        <v>13</v>
+      <c r="G9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="n">
         <v>8386582</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>0.730404786029023</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>11482101.6515995</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>3095519.65159946</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>134317.388692705</v>
       </c>
-      <c r="F10" t="s">
-        <v>14</v>
+      <c r="G10" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="n">
         <v>5365237</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>0.446791544859786</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>12008367.3510065</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>6643130.35100649</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>273310.525668186</v>
       </c>
-      <c r="F11" t="s">
-        <v>15</v>
+      <c r="G11" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -635,36 +716,57 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="n">
         <v>101400750</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" t="n">
         <v>0.885416311072297</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" t="n">
         <v>114523245.993963</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="n">
         <v>13122495.9939631</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="n">
         <v>324868.541667736</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="n">
         <v>0.0247566119903705</v>
       </c>
     </row>
@@ -699,302 +801,335 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="I1" t="s">
-        <v>19</v>
+        <v>34</v>
+      </c>
+      <c r="J1" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="n">
         <v>10012517</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>10012517</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="e">
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="e">
         <v>#NUM!</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>10012517</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="n">
         <v>10283286</v>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>0.998326294976578</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>10300526.0421807</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>17240.0421806891</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>1941.39800536844</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>0.112609817599115</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>10305664</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>-5137.95781931095</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>-0.05</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="n">
         <v>10981123</v>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>0.995761637387273</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>11027863.0825875</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>46740.0825875085</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>5063.30070348638</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>0.108328877981905</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>11033560</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>-5696.91741249152</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>-0.052</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
         <v>11837901</v>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>0.991073866095176</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>11944519.3794094</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>106618.379409375</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>5623.5142744777</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>0.0527443233111386</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>11953731</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>-9211.62059062533</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>-0.077</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="n">
         <v>12490512</v>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>0.981641268511941</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>12724110.5286193</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>233598.528619304</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>8979.08990993114</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>0.0384381269993544</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>12738347</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>-14236.4713806957</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>-0.112</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="n">
         <v>11561287</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>0.963171627924413</v>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>12003350.8720704</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>442063.872070435</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>12089.1055006381</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>0.0273469655957588</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>12057898</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>-54547.1279295646</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>-0.452</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="n">
         <v>10710159</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>0.925130984191426</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>11576910.9272249</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>866751.927224856</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>23680.3493127652</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>0.0273207922231962</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>11630041</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>-53130.0727751441</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>-0.457</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="n">
         <v>9772146</v>
       </c>
-      <c r="B9" t="n">
+      <c r="C9" t="n">
         <v>0.853986174753088</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>11442979.159265</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>1670833.15926497</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>63393.4137139695</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>0.0379411991930166</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>11511377</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>-68397.8407350276</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>-0.594</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="n">
         <v>8386582</v>
       </c>
-      <c r="B10" t="n">
+      <c r="C10" t="n">
         <v>0.730404786029023</v>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>11482101.6515995</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>3095519.65159946</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>134317.388692705</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>0.0433909016288438</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>11554417</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>-72315.3484005351</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>-0.626</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="n">
         <v>5365237</v>
       </c>
-      <c r="B11" t="n">
+      <c r="C11" t="n">
         <v>0.446791544859786</v>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>12008367.3510065</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>6643130.35100649</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>273310.525668186</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>0.041141827907498</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>12061902</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>-53534.6489935089</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>-0.444</v>
       </c>
     </row>

</xml_diff>